<commit_message>
icnrease mem per cpu for GPU jobs
</commit_message>
<xml_diff>
--- a/test_data/norfolk_coastal_flooding/full_benchmarking_experiment_uva_test.xlsx
+++ b/test_data/norfolk_coastal_flooding/full_benchmarking_experiment_uva_test.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\dcl3nd\dev\TRITON-SWMM_toolkit\test_data\norfolk_coastal_flooding\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26ACF394-B438-472B-A9A9-70FD951C5DD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42906913-2F3B-4389-A6BF-243A87459A12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="4185" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="26">
   <si>
     <t>hardware_utilization_strategy</t>
   </si>
@@ -108,6 +108,9 @@
   </si>
   <si>
     <t>serial</t>
+  </si>
+  <si>
+    <t>mem_gb_per_cpu</t>
   </si>
 </sst>
 </file>
@@ -380,7 +383,49 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="1">
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF3F3F76"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFCC99"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FF000000"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF000000"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF000000"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF000000"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -394,9 +439,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:L42" totalsRowShown="0">
-  <autoFilter ref="A1:L42" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
-  <tableColumns count="12">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:M42" totalsRowShown="0">
+  <autoFilter ref="A1:M42" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+  <tableColumns count="13">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="hardware_utilization_strategy"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="device"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="run_mode"/>
@@ -405,6 +450,7 @@
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="n_omp_threads"/>
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="n_gpus"/>
     <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="hpc_ensemble_partition"/>
+    <tableColumn id="9" xr3:uid="{26339B98-C3B5-4C3B-9409-F4B744B2B94C}" name="mem_gb_per_cpu" dataDxfId="0"/>
     <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="total_OpenMP_threads"/>
     <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="total_devices"/>
     <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="devices_per_node"/>
@@ -702,7 +748,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:L42"/>
+  <dimension ref="A1:M42"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="29.85546875" style="20" bestFit="1" customWidth="1"/>
@@ -712,13 +758,14 @@
     <col min="5" max="5" width="22.42578125" style="22" bestFit="1" customWidth="1"/>
     <col min="6" max="7" width="28.28515625" style="22" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="28.28515625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="24.7109375" style="22" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="19" style="22" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="19.85546875" style="22" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="28.28515625" customWidth="1"/>
+    <col min="10" max="10" width="24.7109375" style="22" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="19" style="22" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="19.85546875" style="22" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -743,20 +790,23 @@
       <c r="H1" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="5" t="s">
-        <v>8</v>
+      <c r="I1" s="4" t="s">
+        <v>25</v>
       </c>
       <c r="J1" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="K1" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="6" t="s">
+      <c r="L1" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="M1" s="2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
         <v>12</v>
       </c>
@@ -781,24 +831,27 @@
       <c r="H2" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="I2" s="12">
-        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>1</v>
+      <c r="I2" s="11">
+        <v>8</v>
       </c>
       <c r="J2" s="12">
-        <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>1</v>
-      </c>
-      <c r="K2" s="13">
-        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>1</v>
-      </c>
-      <c r="L2" t="b">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>1</v>
+      </c>
+      <c r="K2" s="12">
+        <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
+        <v>1</v>
+      </c>
+      <c r="L2" s="13">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+      <c r="M2" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
         <v>12</v>
       </c>
@@ -823,24 +876,27 @@
       <c r="H3" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="I3" s="12">
-        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>2</v>
+      <c r="I3" s="11">
+        <v>8</v>
       </c>
       <c r="J3" s="12">
-        <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>2</v>
-      </c>
-      <c r="K3" s="13">
-        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>2</v>
-      </c>
-      <c r="L3" t="b">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>2</v>
+      </c>
+      <c r="K3" s="12">
+        <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
+        <v>2</v>
+      </c>
+      <c r="L3" s="13">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>2</v>
+      </c>
+      <c r="M3" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
         <v>12</v>
       </c>
@@ -865,24 +921,27 @@
       <c r="H4" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="I4" s="12">
+      <c r="I4" s="11">
+        <v>8</v>
+      </c>
+      <c r="J4" s="12">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
         <v>3</v>
       </c>
-      <c r="J4" s="12">
+      <c r="K4" s="12">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
         <v>3</v>
       </c>
-      <c r="K4" s="13">
+      <c r="L4" s="13">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
         <v>3</v>
       </c>
-      <c r="L4" t="b">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M4" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
         <v>12</v>
       </c>
@@ -907,24 +966,27 @@
       <c r="H5" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="I5" s="12">
+      <c r="I5" s="11">
+        <v>8</v>
+      </c>
+      <c r="J5" s="12">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
         <v>4</v>
       </c>
-      <c r="J5" s="12">
+      <c r="K5" s="12">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
         <v>4</v>
       </c>
-      <c r="K5" s="13">
+      <c r="L5" s="13">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
         <v>4</v>
       </c>
-      <c r="L5" t="b">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M5" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
         <v>12</v>
       </c>
@@ -949,24 +1011,27 @@
       <c r="H6" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="I6" s="12">
+      <c r="I6" s="11">
+        <v>8</v>
+      </c>
+      <c r="J6" s="12">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
         <v>5</v>
       </c>
-      <c r="J6" s="12">
+      <c r="K6" s="12">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
         <v>5</v>
       </c>
-      <c r="K6" s="13">
+      <c r="L6" s="13">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
         <v>5</v>
       </c>
-      <c r="L6" t="b">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M6" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
         <v>12</v>
       </c>
@@ -991,24 +1056,27 @@
       <c r="H7" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="I7" s="12">
+      <c r="I7" s="11">
+        <v>8</v>
+      </c>
+      <c r="J7" s="12">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
         <v>6</v>
       </c>
-      <c r="J7" s="12">
+      <c r="K7" s="12">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
         <v>6</v>
       </c>
-      <c r="K7" s="13">
+      <c r="L7" s="13">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
         <v>6</v>
       </c>
-      <c r="L7" t="b">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M7" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
         <v>12</v>
       </c>
@@ -1033,24 +1101,27 @@
       <c r="H8" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="I8" s="12">
+      <c r="I8" s="11">
+        <v>8</v>
+      </c>
+      <c r="J8" s="12">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
         <v>7</v>
       </c>
-      <c r="J8" s="12">
+      <c r="K8" s="12">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
         <v>7</v>
       </c>
-      <c r="K8" s="13">
+      <c r="L8" s="13">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
         <v>7</v>
       </c>
-      <c r="L8" t="b">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M8" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="7" t="s">
         <v>12</v>
       </c>
@@ -1075,24 +1146,27 @@
       <c r="H9" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="I9" s="12">
-        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+      <c r="I9" s="11">
         <v>8</v>
       </c>
       <c r="J9" s="12">
-        <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>8</v>
-      </c>
-      <c r="K9" s="13">
-        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>8</v>
-      </c>
-      <c r="L9" t="b">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>8</v>
+      </c>
+      <c r="K9" s="12">
+        <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
+        <v>8</v>
+      </c>
+      <c r="L9" s="13">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>8</v>
+      </c>
+      <c r="M9" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="7" t="s">
         <v>12</v>
       </c>
@@ -1117,24 +1191,27 @@
       <c r="H10" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="I10" s="12">
-        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>16</v>
+      <c r="I10" s="11">
+        <v>8</v>
       </c>
       <c r="J10" s="12">
-        <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>16</v>
-      </c>
-      <c r="K10" s="13">
-        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>8</v>
-      </c>
-      <c r="L10" t="b">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>16</v>
+      </c>
+      <c r="K10" s="12">
+        <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
+        <v>16</v>
+      </c>
+      <c r="L10" s="13">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>8</v>
+      </c>
+      <c r="M10" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
         <v>14</v>
       </c>
@@ -1159,24 +1236,27 @@
       <c r="H11" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="I11" s="12">
+      <c r="I11" s="11">
+        <v>2</v>
+      </c>
+      <c r="J11" s="12">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
         <v>4</v>
       </c>
-      <c r="J11" s="12">
+      <c r="K11" s="12">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
         <v>4</v>
       </c>
-      <c r="K11" s="13">
+      <c r="L11" s="13">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
         <v>4</v>
       </c>
-      <c r="L11" t="b">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M11" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="16" t="s">
         <v>14</v>
       </c>
@@ -1201,24 +1281,27 @@
       <c r="H12" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="I12" s="12">
-        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>8</v>
+      <c r="I12" s="11">
+        <v>2</v>
       </c>
       <c r="J12" s="12">
-        <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>8</v>
-      </c>
-      <c r="K12" s="19">
-        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>8</v>
-      </c>
-      <c r="L12" t="b">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>8</v>
+      </c>
+      <c r="K12" s="12">
+        <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
+        <v>8</v>
+      </c>
+      <c r="L12" s="19">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>8</v>
+      </c>
+      <c r="M12" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="14" t="s">
         <v>14</v>
       </c>
@@ -1243,24 +1326,27 @@
       <c r="H13" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="I13" s="12">
-        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>8</v>
+      <c r="I13" s="11">
+        <v>2</v>
       </c>
       <c r="J13" s="12">
-        <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>8</v>
-      </c>
-      <c r="K13" s="19">
-        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>8</v>
-      </c>
-      <c r="L13" t="b">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>8</v>
+      </c>
+      <c r="K13" s="12">
+        <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
+        <v>8</v>
+      </c>
+      <c r="L13" s="19">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>8</v>
+      </c>
+      <c r="M13" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="14" t="s">
         <v>14</v>
       </c>
@@ -1285,24 +1371,27 @@
       <c r="H14" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="I14" s="12">
-        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>16</v>
+      <c r="I14" s="11">
+        <v>2</v>
       </c>
       <c r="J14" s="12">
-        <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>16</v>
-      </c>
-      <c r="K14" s="19">
-        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>16</v>
-      </c>
-      <c r="L14" t="b">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>16</v>
+      </c>
+      <c r="K14" s="12">
+        <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
+        <v>16</v>
+      </c>
+      <c r="L14" s="19">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>16</v>
+      </c>
+      <c r="M14" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="14" t="s">
         <v>14</v>
       </c>
@@ -1327,24 +1416,27 @@
       <c r="H15" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="I15" s="12">
-        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>16</v>
+      <c r="I15" s="11">
+        <v>2</v>
       </c>
       <c r="J15" s="12">
-        <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>16</v>
-      </c>
-      <c r="K15" s="19">
-        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>16</v>
-      </c>
-      <c r="L15" t="b">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>16</v>
+      </c>
+      <c r="K15" s="12">
+        <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
+        <v>16</v>
+      </c>
+      <c r="L15" s="19">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>16</v>
+      </c>
+      <c r="M15" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="14" t="s">
         <v>14</v>
       </c>
@@ -1369,24 +1461,27 @@
       <c r="H16" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="I16" s="12">
-        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>16</v>
+      <c r="I16" s="11">
+        <v>2</v>
       </c>
       <c r="J16" s="12">
-        <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>16</v>
-      </c>
-      <c r="K16" s="19">
-        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>16</v>
-      </c>
-      <c r="L16" t="b">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>16</v>
+      </c>
+      <c r="K16" s="12">
+        <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
+        <v>16</v>
+      </c>
+      <c r="L16" s="19">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>16</v>
+      </c>
+      <c r="M16" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="14" t="s">
         <v>14</v>
       </c>
@@ -1411,24 +1506,27 @@
       <c r="H17" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="I17" s="12">
+      <c r="I17" s="11">
+        <v>2</v>
+      </c>
+      <c r="J17" s="12">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
         <v>32</v>
       </c>
-      <c r="J17" s="12">
+      <c r="K17" s="12">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
         <v>32</v>
       </c>
-      <c r="K17" s="19">
+      <c r="L17" s="19">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
         <v>32</v>
       </c>
-      <c r="L17" t="b">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="18" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M17" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="14" t="s">
         <v>14</v>
       </c>
@@ -1453,24 +1551,27 @@
       <c r="H18" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="I18" s="12">
+      <c r="I18" s="11">
+        <v>2</v>
+      </c>
+      <c r="J18" s="12">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
         <v>32</v>
       </c>
-      <c r="J18" s="12">
+      <c r="K18" s="12">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
         <v>32</v>
       </c>
-      <c r="K18" s="19">
+      <c r="L18" s="19">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
         <v>32</v>
       </c>
-      <c r="L18" t="b">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M18" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="14" t="s">
         <v>14</v>
       </c>
@@ -1495,24 +1596,27 @@
       <c r="H19" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="I19" s="12">
+      <c r="I19" s="11">
+        <v>2</v>
+      </c>
+      <c r="J19" s="12">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
         <v>32</v>
       </c>
-      <c r="J19" s="12">
+      <c r="K19" s="12">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
         <v>32</v>
       </c>
-      <c r="K19" s="19">
+      <c r="L19" s="19">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
         <v>32</v>
       </c>
-      <c r="L19" t="b">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="20" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M19" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="14" t="s">
         <v>14</v>
       </c>
@@ -1537,24 +1641,27 @@
       <c r="H20" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="I20" s="12">
+      <c r="I20" s="11">
+        <v>2</v>
+      </c>
+      <c r="J20" s="12">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
         <v>32</v>
       </c>
-      <c r="J20" s="12">
+      <c r="K20" s="12">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
         <v>32</v>
       </c>
-      <c r="K20" s="19">
+      <c r="L20" s="19">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
         <v>32</v>
       </c>
-      <c r="L20" t="b">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="21" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M20" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="14" t="s">
         <v>14</v>
       </c>
@@ -1579,24 +1686,27 @@
       <c r="H21" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="I21" s="12">
+      <c r="I21" s="11">
+        <v>2</v>
+      </c>
+      <c r="J21" s="12">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
         <v>64</v>
       </c>
-      <c r="J21" s="12">
+      <c r="K21" s="12">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
         <v>64</v>
       </c>
-      <c r="K21" s="19">
+      <c r="L21" s="19">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
         <v>64</v>
       </c>
-      <c r="L21" t="b">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="22" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M21" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="14" t="s">
         <v>14</v>
       </c>
@@ -1621,24 +1731,27 @@
       <c r="H22" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="I22" s="12">
+      <c r="I22" s="11">
+        <v>2</v>
+      </c>
+      <c r="J22" s="12">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
         <v>64</v>
       </c>
-      <c r="J22" s="12">
+      <c r="K22" s="12">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
         <v>64</v>
       </c>
-      <c r="K22" s="19">
+      <c r="L22" s="19">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
         <v>64</v>
       </c>
-      <c r="L22" t="b">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="23" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M22" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="14" t="s">
         <v>14</v>
       </c>
@@ -1663,24 +1776,27 @@
       <c r="H23" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="I23" s="12">
+      <c r="I23" s="11">
+        <v>2</v>
+      </c>
+      <c r="J23" s="12">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
         <v>64</v>
       </c>
-      <c r="J23" s="12">
+      <c r="K23" s="12">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
         <v>64</v>
       </c>
-      <c r="K23" s="19">
+      <c r="L23" s="19">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
         <v>64</v>
       </c>
-      <c r="L23" t="b">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="24" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M23" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="14" t="s">
         <v>14</v>
       </c>
@@ -1705,24 +1821,27 @@
       <c r="H24" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="I24" s="12">
+      <c r="I24" s="11">
+        <v>2</v>
+      </c>
+      <c r="J24" s="12">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
         <v>64</v>
       </c>
-      <c r="J24" s="12">
+      <c r="K24" s="12">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
         <v>64</v>
       </c>
-      <c r="K24" s="19">
+      <c r="L24" s="19">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
         <v>64</v>
       </c>
-      <c r="L24" t="b">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="25" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M24" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="14" t="s">
         <v>14</v>
       </c>
@@ -1747,24 +1866,27 @@
       <c r="H25" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="I25" s="12">
+      <c r="I25" s="11">
+        <v>2</v>
+      </c>
+      <c r="J25" s="12">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
         <v>64</v>
       </c>
-      <c r="J25" s="12">
+      <c r="K25" s="12">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
         <v>64</v>
       </c>
-      <c r="K25" s="19">
+      <c r="L25" s="19">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
         <v>64</v>
       </c>
-      <c r="L25" t="b">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="26" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M25" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="14" t="s">
         <v>14</v>
       </c>
@@ -1789,24 +1911,27 @@
       <c r="H26" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="I26" s="12">
+      <c r="I26" s="11">
+        <v>2</v>
+      </c>
+      <c r="J26" s="12">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
         <v>128</v>
       </c>
-      <c r="J26" s="12">
+      <c r="K26" s="12">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
         <v>128</v>
       </c>
-      <c r="K26" s="19">
+      <c r="L26" s="19">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
         <v>64</v>
       </c>
-      <c r="L26" t="b">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="27" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M26" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="14" t="s">
         <v>14</v>
       </c>
@@ -1831,24 +1956,27 @@
       <c r="H27" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="I27" s="12">
+      <c r="I27" s="11">
+        <v>2</v>
+      </c>
+      <c r="J27" s="12">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
         <v>128</v>
       </c>
-      <c r="J27" s="12">
+      <c r="K27" s="12">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
         <v>128</v>
       </c>
-      <c r="K27" s="19">
+      <c r="L27" s="19">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
         <v>64</v>
       </c>
-      <c r="L27" t="b">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="28" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M27" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="14" t="s">
         <v>14</v>
       </c>
@@ -1873,24 +2001,27 @@
       <c r="H28" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="I28" s="12">
+      <c r="I28" s="11">
+        <v>2</v>
+      </c>
+      <c r="J28" s="12">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
         <v>128</v>
       </c>
-      <c r="J28" s="12">
+      <c r="K28" s="12">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
         <v>128</v>
       </c>
-      <c r="K28" s="19">
+      <c r="L28" s="19">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
         <v>64</v>
       </c>
-      <c r="L28" t="b">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="29" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M28" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="14" t="s">
         <v>14</v>
       </c>
@@ -1915,24 +2046,27 @@
       <c r="H29" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="I29" s="12">
+      <c r="I29" s="11">
+        <v>2</v>
+      </c>
+      <c r="J29" s="12">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
         <v>128</v>
       </c>
-      <c r="J29" s="12">
+      <c r="K29" s="12">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
         <v>128</v>
       </c>
-      <c r="K29" s="19">
+      <c r="L29" s="19">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
         <v>64</v>
       </c>
-      <c r="L29" t="b">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="30" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M29" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="14" t="s">
         <v>14</v>
       </c>
@@ -1957,24 +2091,27 @@
       <c r="H30" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="I30" s="12">
+      <c r="I30" s="11">
+        <v>2</v>
+      </c>
+      <c r="J30" s="12">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
         <v>128</v>
       </c>
-      <c r="J30" s="12">
+      <c r="K30" s="12">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
         <v>128</v>
       </c>
-      <c r="K30" s="19">
+      <c r="L30" s="19">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
         <v>64</v>
       </c>
-      <c r="L30" t="b">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="31" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M30" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="14" t="s">
         <v>14</v>
       </c>
@@ -1999,24 +2136,27 @@
       <c r="H31" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="I31" s="12">
+      <c r="I31" s="11">
+        <v>2</v>
+      </c>
+      <c r="J31" s="12">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
         <v>128</v>
       </c>
-      <c r="J31" s="12">
+      <c r="K31" s="12">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
         <v>128</v>
       </c>
-      <c r="K31" s="19">
+      <c r="L31" s="19">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
         <v>64</v>
       </c>
-      <c r="L31" t="b">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="32" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M31" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="14" t="s">
         <v>19</v>
       </c>
@@ -2041,24 +2181,27 @@
       <c r="H32" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="I32" s="12">
-        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+      <c r="I32" s="11">
         <v>2</v>
       </c>
       <c r="J32" s="12">
-        <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>2</v>
-      </c>
-      <c r="K32" s="19">
-        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>2</v>
-      </c>
-      <c r="L32" t="b">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="33" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>2</v>
+      </c>
+      <c r="K32" s="12">
+        <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
+        <v>2</v>
+      </c>
+      <c r="L32" s="19">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>2</v>
+      </c>
+      <c r="M32" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="14" t="s">
         <v>19</v>
       </c>
@@ -2083,24 +2226,27 @@
       <c r="H33" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="I33" s="12">
+      <c r="I33" s="11">
+        <v>2</v>
+      </c>
+      <c r="J33" s="12">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
         <v>4</v>
       </c>
-      <c r="J33" s="12">
+      <c r="K33" s="12">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
         <v>4</v>
       </c>
-      <c r="K33" s="19">
+      <c r="L33" s="19">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
         <v>4</v>
       </c>
-      <c r="L33" t="b">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="34" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M33" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="14" t="s">
         <v>19</v>
       </c>
@@ -2125,24 +2271,27 @@
       <c r="H34" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="I34" s="12">
-        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>8</v>
+      <c r="I34" s="11">
+        <v>2</v>
       </c>
       <c r="J34" s="12">
-        <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>8</v>
-      </c>
-      <c r="K34" s="19">
-        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>8</v>
-      </c>
-      <c r="L34" t="b">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="35" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>8</v>
+      </c>
+      <c r="K34" s="12">
+        <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
+        <v>8</v>
+      </c>
+      <c r="L34" s="19">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>8</v>
+      </c>
+      <c r="M34" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="14" t="s">
         <v>19</v>
       </c>
@@ -2167,24 +2316,27 @@
       <c r="H35" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="I35" s="12">
-        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>16</v>
+      <c r="I35" s="11">
+        <v>2</v>
       </c>
       <c r="J35" s="12">
-        <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>16</v>
-      </c>
-      <c r="K35" s="19">
-        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>16</v>
-      </c>
-      <c r="L35" t="b">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="36" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>16</v>
+      </c>
+      <c r="K35" s="12">
+        <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
+        <v>16</v>
+      </c>
+      <c r="L35" s="19">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>16</v>
+      </c>
+      <c r="M35" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="14" t="s">
         <v>21</v>
       </c>
@@ -2209,24 +2361,27 @@
       <c r="H36" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="I36" s="12">
-        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+      <c r="I36" s="11">
         <v>2</v>
       </c>
       <c r="J36" s="12">
-        <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>2</v>
-      </c>
-      <c r="K36" s="19">
-        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>2</v>
-      </c>
-      <c r="L36" t="b">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="37" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>2</v>
+      </c>
+      <c r="K36" s="12">
+        <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
+        <v>2</v>
+      </c>
+      <c r="L36" s="19">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>2</v>
+      </c>
+      <c r="M36" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="14" t="s">
         <v>21</v>
       </c>
@@ -2251,24 +2406,27 @@
       <c r="H37" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="I37" s="12">
+      <c r="I37" s="11">
+        <v>2</v>
+      </c>
+      <c r="J37" s="12">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
         <v>4</v>
       </c>
-      <c r="J37" s="12">
+      <c r="K37" s="12">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
         <v>4</v>
       </c>
-      <c r="K37" s="19">
+      <c r="L37" s="19">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
         <v>4</v>
       </c>
-      <c r="L37" t="b">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="38" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M37" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="14" t="s">
         <v>21</v>
       </c>
@@ -2293,24 +2451,27 @@
       <c r="H38" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="I38" s="12">
-        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>8</v>
+      <c r="I38" s="11">
+        <v>2</v>
       </c>
       <c r="J38" s="12">
-        <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>8</v>
-      </c>
-      <c r="K38" s="19">
-        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>8</v>
-      </c>
-      <c r="L38" t="b">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="39" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>8</v>
+      </c>
+      <c r="K38" s="12">
+        <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
+        <v>8</v>
+      </c>
+      <c r="L38" s="19">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>8</v>
+      </c>
+      <c r="M38" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="14" t="s">
         <v>21</v>
       </c>
@@ -2335,24 +2496,27 @@
       <c r="H39" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="I39" s="12">
-        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>16</v>
+      <c r="I39" s="11">
+        <v>2</v>
       </c>
       <c r="J39" s="12">
-        <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>16</v>
-      </c>
-      <c r="K39" s="19">
-        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>16</v>
-      </c>
-      <c r="L39" t="b">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="40" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>16</v>
+      </c>
+      <c r="K39" s="12">
+        <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
+        <v>16</v>
+      </c>
+      <c r="L39" s="19">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>16</v>
+      </c>
+      <c r="M39" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="14" t="s">
         <v>21</v>
       </c>
@@ -2377,24 +2541,27 @@
       <c r="H40" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="I40" s="12">
+      <c r="I40" s="11">
+        <v>2</v>
+      </c>
+      <c r="J40" s="12">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
         <v>32</v>
       </c>
-      <c r="J40" s="12">
+      <c r="K40" s="12">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
         <v>32</v>
       </c>
-      <c r="K40" s="19">
+      <c r="L40" s="19">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
         <v>32</v>
       </c>
-      <c r="L40" t="b">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="41" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M40" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="14" t="s">
         <v>21</v>
       </c>
@@ -2419,24 +2586,27 @@
       <c r="H41" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="I41" s="12">
+      <c r="I41" s="11">
+        <v>2</v>
+      </c>
+      <c r="J41" s="12">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
         <v>64</v>
       </c>
-      <c r="J41" s="12">
+      <c r="K41" s="12">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
         <v>64</v>
       </c>
-      <c r="K41" s="19">
+      <c r="L41" s="19">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
         <v>64</v>
       </c>
-      <c r="L41" t="b">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="42" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M41" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="14" t="s">
         <v>23</v>
       </c>
@@ -2461,19 +2631,22 @@
       <c r="H42" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="I42" s="12">
-        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>1</v>
+      <c r="I42" s="11">
+        <v>2</v>
       </c>
       <c r="J42" s="12">
-        <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>1</v>
-      </c>
-      <c r="K42" s="19">
-        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>1</v>
-      </c>
-      <c r="L42" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>1</v>
+      </c>
+      <c r="K42" s="12">
+        <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
+        <v>1</v>
+      </c>
+      <c r="L42" s="19">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+      <c r="M42" t="b">
         <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
         <v>1</v>
       </c>

</xml_diff>